<commit_message>
Publica dados para o portal de visualizacao
</commit_message>
<xml_diff>
--- a/dados_publicados/antecipacao.xlsx
+++ b/dados_publicados/antecipacao.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://daterrinhaalimentoscombr.sharepoint.com/sites/DT-FinanceiroCP/DADOS/CONFIRMAÇÂO DE ENTREGA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="972" documentId="8_{E176FAEE-370F-4BDD-B645-D2812466DC45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7FF89A8-4FC6-47EA-B7F1-DDBB63B38256}"/>
+  <xr:revisionPtr revIDLastSave="985" documentId="8_{E176FAEE-370F-4BDD-B645-D2812466DC45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0ED32FF-85FB-4B2C-BF4E-3B1EA3A43032}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-45" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Linha do tempo." sheetId="10" r:id="rId1"/>
@@ -23,8 +23,8 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId5"/>
-    <pivotCache cacheId="1" r:id="rId6"/>
+    <pivotCache cacheId="10" r:id="rId5"/>
+    <pivotCache cacheId="19" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="39">
   <si>
     <t>Mês</t>
   </si>
@@ -158,19 +158,33 @@
   <si>
     <t>Agpsto</t>
   </si>
+  <si>
+    <t>Setembro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOGUBER GESTAO EM TRANSPORTES LTDA </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -304,10 +318,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -322,57 +336,63 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="10" fontId="2" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="3" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" pivotButton="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" pivotButton="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -380,20 +400,237 @@
     <xf numFmtId="10" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" pivotButton="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" pivotButton="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="46">
+  <dxfs count="75">
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="13"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="13"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="13"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="13"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="13"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="13"/>
+      </font>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="13"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="15"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <sz val="15"/>
@@ -1809,6 +2046,1017 @@
           </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="17"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="18"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="19"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent2"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="6.008712633318293E-3"/>
+              <c:y val="0"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="20"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent2"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="7.0101647388713271E-3"/>
+              <c:y val="0"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="21"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent2"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="9.0130689499773944E-3"/>
+              <c:y val="0"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="22"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent2"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="1.201742526663655E-2"/>
+              <c:y val="-3.3815186426850428E-3"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="23"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent2"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="3.0043563166592293E-3"/>
+              <c:y val="0"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="24"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent2"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="8.0116168444242693E-3"/>
+              <c:y val="0"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="25"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent2"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="1.4020329477742727E-2"/>
+              <c:y val="-3.3815186426851668E-3"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="26"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="27"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent3"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="2.0762862055492274E-2"/>
+              <c:y val="0"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="28"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent3"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="1.880961977697165E-2"/>
+              <c:y val="0"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="29"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent3"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="2.4557182718090837E-2"/>
+              <c:y val="-3.3815186426850428E-3"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="30"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent3"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="2.7138484661026131E-2"/>
+              <c:y val="0"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="31"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent3"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="1.9705315956827313E-2"/>
+              <c:y val="0"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="32"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent3"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="1.612253123740414E-2"/>
+              <c:y val="7.5011709505046755E-3"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="33"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent3"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="2.6031288675666182E-2"/>
+              <c:y val="0"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
       <c:layout/>
@@ -1900,9 +3148,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Linha do tempo.'!$A$4:$A$11</c:f>
+              <c:f>'Linha do tempo.'!$A$4:$A$13</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>Janeiro</c:v>
                 </c:pt>
@@ -1924,15 +3172,21 @@
                 <c:pt idx="6">
                   <c:v>Julho</c:v>
                 </c:pt>
+                <c:pt idx="7">
+                  <c:v>Agosto</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Agpsto</c:v>
+                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Linha do tempo.'!$B$4:$B$11</c:f>
+              <c:f>'Linha do tempo.'!$B$4:$B$13</c:f>
               <c:numCache>
                 <c:formatCode>_("R$"* #,##0.00_);_("R$"* \(#,##0.00\);_("R$"* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>114169.85</c:v>
                 </c:pt>
@@ -1953,6 +3207,12 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>176023.93999999997</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>232778.93999999997</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>11041.27</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2334,9 +3594,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Linha do tempo.'!$A$4:$A$11</c:f>
+              <c:f>'Linha do tempo.'!$A$4:$A$13</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>Janeiro</c:v>
                 </c:pt>
@@ -2358,15 +3618,21 @@
                 <c:pt idx="6">
                   <c:v>Julho</c:v>
                 </c:pt>
+                <c:pt idx="7">
+                  <c:v>Agosto</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Agpsto</c:v>
+                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Linha do tempo.'!$C$4:$C$11</c:f>
+              <c:f>'Linha do tempo.'!$C$4:$C$13</c:f>
               <c:numCache>
                 <c:formatCode>_("R$"* #,##0.00_);_("R$"* \(#,##0.00\);_("R$"* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>4325.51</c:v>
                 </c:pt>
@@ -2387,6 +3653,12 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>5496.14</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5529.87</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>436.23</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2768,9 +4040,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Linha do tempo.'!$A$4:$A$11</c:f>
+              <c:f>'Linha do tempo.'!$A$4:$A$13</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>Janeiro</c:v>
                 </c:pt>
@@ -2792,15 +4064,21 @@
                 <c:pt idx="6">
                   <c:v>Julho</c:v>
                 </c:pt>
+                <c:pt idx="7">
+                  <c:v>Agosto</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Agpsto</c:v>
+                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Linha do tempo.'!$D$4:$D$11</c:f>
+              <c:f>'Linha do tempo.'!$D$4:$D$13</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>4.3776150077792307E-2</c:v>
                 </c:pt>
@@ -2821,6 +4099,12 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>4.5113735997973359E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3.603415173702252E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3.6166276882344799E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5266,19 +6550,19 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>624840</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>31431</xdr:rowOff>
+      <xdr:colOff>514350</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>115251</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
-      <xdr:colOff>447675</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:colOff>331470</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>78105</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Gráfico 2">
+        <xdr:cNvPr id="2" name="Gráfico 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D239CD25-79B6-7AE7-B749-32F2617D4B69}"/>
@@ -5343,14 +6627,18 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Daterrinha68" refreshedDate="46253.740368634259" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="101" xr:uid="{5E4BBC87-83C7-4098-86BE-C7579885E474}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Daterrinha68" refreshedDate="46297.453520254632" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="115" xr:uid="{5E4BBC87-83C7-4098-86BE-C7579885E474}">
   <cacheSource type="worksheet">
     <worksheetSource name="Tabela1[[Mês]:[Ganha por %]]"/>
   </cacheSource>
   <cacheFields count="4">
     <cacheField name="Mês" numFmtId="14">
-      <sharedItems count="7">
+      <sharedItems count="9">
         <s v="Janeiro"/>
         <s v="Fevereiro"/>
         <s v="Março"/>
@@ -5358,12 +6646,14 @@
         <s v="Maio"/>
         <s v="Junho"/>
         <s v="Julho"/>
+        <s v="Agosto"/>
+        <s v="Agpsto"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Valor líquido" numFmtId="44">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="64.680000000000007" maxValue="68938.86"/>
+    <cacheField name="Valor líquido" numFmtId="165">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="64.680000000000007" maxValue="108896.46"/>
     </cacheField>
-    <cacheField name="Desconto Financeiro" numFmtId="44">
+    <cacheField name="Desconto Financeiro" numFmtId="165">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1.29" maxValue="3207.6"/>
     </cacheField>
     <cacheField name="Ganha por %" numFmtId="10">
@@ -5379,19 +6669,19 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Daterrinha68" refreshedDate="46253.741340624998" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="101" xr:uid="{40DCFBB4-BCE6-447B-8E94-DDE8F3337F4A}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Daterrinha68" refreshedDate="46297.46620023148" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="129" xr:uid="{40DCFBB4-BCE6-447B-8E94-DDE8F3337F4A}">
   <cacheSource type="worksheet">
     <worksheetSource name="Tabela1"/>
   </cacheSource>
   <cacheFields count="8">
     <cacheField name="L.P" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="10"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="14"/>
     </cacheField>
     <cacheField name="Duplicata" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1281925" maxValue="1562198"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1281925" maxValue="1611752"/>
     </cacheField>
     <cacheField name="Favorecido" numFmtId="0">
-      <sharedItems count="27">
+      <sharedItems count="30">
         <s v="FORT TAPE INDUSTRIA E COMERCIO DE MATERIAIS ADESIVOS LTDA "/>
         <s v="JM CONFECCOES EIRELI"/>
         <s v="FWSG COMERCIO E SERVICOS LTDA - ME - CONSULTORIA "/>
@@ -5400,6 +6690,9 @@
         <s v="DU PRATA ALIMENTOS LTDA - FORN: DU PRATA ALIMENTOS "/>
         <s v="GROSS PACK INDUSTRIA E COMERCIO LTDA"/>
         <s v="JNBM - CONDIMENTOS E ESPECIARIAS LTDA"/>
+        <s v="FLAVIA MEDEIROS SILVA - SERVICOS LOGISTICOS "/>
+        <s v="LOGUBER GESTAO EM TRANSPORTES LTDA "/>
+        <s v=" FLAVIA MEDEIROS SILVA - SERVICOS LOGISTICOS " u="1"/>
         <s v="JM CONFECCOES EIRELI " u="1"/>
         <s v="GROSS PACK INDUSTRIA E COMERCIO LTDA " u="1"/>
         <s v="175177 - DESPACHOS ENCOMENDAS E CARGAS LOGISTICA LTDA - DESPESAS DE CORRESPONDENCIA - Nº 152" u="1"/>
@@ -5422,10 +6715,10 @@
       </sharedItems>
     </cacheField>
     <cacheField name="Vencimento" numFmtId="14">
-      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-01-05T00:00:00" maxDate="2026-08-01T00:00:00"/>
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-01-05T00:00:00" maxDate="2026-10-01T00:00:00"/>
     </cacheField>
     <cacheField name="Mês" numFmtId="14">
-      <sharedItems count="7">
+      <sharedItems count="10">
         <s v="Janeiro"/>
         <s v="Fevereiro"/>
         <s v="Março"/>
@@ -5433,13 +6726,16 @@
         <s v="Maio"/>
         <s v="Junho"/>
         <s v="Julho"/>
+        <s v="Agosto"/>
+        <s v="Agpsto"/>
+        <s v="Setembro"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Valor líquido" numFmtId="44">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="64.680000000000007" maxValue="68938.86"/>
+    <cacheField name="Valor líquido" numFmtId="165">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="64.680000000000007" maxValue="112933.07"/>
     </cacheField>
-    <cacheField name="Desconto Financeiro" numFmtId="44">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1.29" maxValue="3207.6"/>
+    <cacheField name="Desconto Financeiro" numFmtId="165">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1.29" maxValue="8181.49"/>
     </cacheField>
     <cacheField name="Ganha por %" numFmtId="10">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1.3098800431168847E-3" maxValue="9.7321945423339801E-2"/>
@@ -5454,7 +6750,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="101">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="115">
   <r>
     <x v="0"/>
     <n v="9724.93"/>
@@ -6061,11 +7357,95 @@
     <n v="281.81"/>
     <n v="9.0527113803770654E-2"/>
   </r>
+  <r>
+    <x v="7"/>
+    <n v="19206.62"/>
+    <n v="604.76"/>
+    <n v="3.1487060190705081E-2"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <n v="28327.01"/>
+    <n v="494.02"/>
+    <n v="1.743989217358274E-2"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <n v="661.87"/>
+    <n v="10.63"/>
+    <n v="1.60605556982489E-2"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <n v="651.97"/>
+    <n v="20.53"/>
+    <n v="3.1489178949951686E-2"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <n v="633.61"/>
+    <n v="38.89"/>
+    <n v="6.1378450466375217E-2"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <n v="1742.01"/>
+    <n v="27.99"/>
+    <n v="1.6067645995143539E-2"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <n v="3025.81"/>
+    <n v="139.19"/>
+    <n v="4.6000905542648088E-2"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <n v="4326"/>
+    <n v="199"/>
+    <n v="4.6000924641701343E-2"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <n v="37643.589999999997"/>
+    <n v="98.81"/>
+    <n v="2.6248824833125643E-3"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <n v="108896.46"/>
+    <n v="1749.54"/>
+    <n v="1.6066086996767388E-2"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <n v="29137.15"/>
+    <n v="2110.85"/>
+    <n v="7.2445314658434332E-2"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <n v="731.65"/>
+    <n v="33.35"/>
+    <n v="4.5581903915806743E-2"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <n v="3121.87"/>
+    <n v="178.13"/>
+    <n v="5.7058750044044114E-2"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <n v="5714.59"/>
+    <n v="260.41000000000003"/>
+    <n v="4.5569323433527167E-2"/>
+  </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="101">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="129">
   <r>
     <n v="1"/>
     <n v="1281925"/>
@@ -7076,15 +8456,295 @@
     <n v="281.81"/>
     <n v="9.0527113803770654E-2"/>
   </r>
+  <r>
+    <n v="1"/>
+    <n v="1566269"/>
+    <x v="4"/>
+    <d v="2026-08-07T00:00:00"/>
+    <x v="7"/>
+    <n v="19206.62"/>
+    <n v="604.76"/>
+    <n v="3.1487060190705081E-2"/>
+  </r>
+  <r>
+    <n v="1"/>
+    <n v="1576713"/>
+    <x v="8"/>
+    <d v="2026-08-17T00:00:00"/>
+    <x v="7"/>
+    <n v="28327.01"/>
+    <n v="494.02"/>
+    <n v="1.743989217358274E-2"/>
+  </r>
+  <r>
+    <n v="6"/>
+    <n v="1562728"/>
+    <x v="1"/>
+    <d v="2026-08-18T00:00:00"/>
+    <x v="8"/>
+    <n v="661.87"/>
+    <n v="10.63"/>
+    <n v="1.60605556982489E-2"/>
+  </r>
+  <r>
+    <n v="6"/>
+    <n v="1562729"/>
+    <x v="1"/>
+    <d v="2026-08-18T00:00:00"/>
+    <x v="8"/>
+    <n v="651.97"/>
+    <n v="20.53"/>
+    <n v="3.1489178949951686E-2"/>
+  </r>
+  <r>
+    <n v="6"/>
+    <n v="1562730"/>
+    <x v="1"/>
+    <d v="2026-08-18T00:00:00"/>
+    <x v="8"/>
+    <n v="633.61"/>
+    <n v="38.89"/>
+    <n v="6.1378450466375217E-2"/>
+  </r>
+  <r>
+    <n v="6"/>
+    <n v="1578292"/>
+    <x v="1"/>
+    <d v="2026-08-18T00:00:00"/>
+    <x v="8"/>
+    <n v="1742.01"/>
+    <n v="27.99"/>
+    <n v="1.6067645995143539E-2"/>
+  </r>
+  <r>
+    <n v="14"/>
+    <n v="1578295"/>
+    <x v="1"/>
+    <d v="2026-08-18T00:00:00"/>
+    <x v="8"/>
+    <n v="3025.81"/>
+    <n v="139.19"/>
+    <n v="4.6000905542648088E-2"/>
+  </r>
+  <r>
+    <n v="1"/>
+    <n v="1578293"/>
+    <x v="1"/>
+    <d v="2026-08-18T00:00:00"/>
+    <x v="8"/>
+    <n v="4326"/>
+    <n v="199"/>
+    <n v="4.6000924641701343E-2"/>
+  </r>
+  <r>
+    <n v="14"/>
+    <n v="1540990"/>
+    <x v="5"/>
+    <d v="2026-08-18T00:00:00"/>
+    <x v="7"/>
+    <n v="37643.589999999997"/>
+    <n v="98.81"/>
+    <n v="2.6248824833125643E-3"/>
+  </r>
+  <r>
+    <n v="14"/>
+    <n v="1554474"/>
+    <x v="5"/>
+    <d v="2026-08-18T00:00:00"/>
+    <x v="7"/>
+    <n v="108896.46"/>
+    <n v="1749.54"/>
+    <n v="1.6066086996767388E-2"/>
+  </r>
+  <r>
+    <n v="14"/>
+    <n v="1581223"/>
+    <x v="5"/>
+    <d v="2026-08-21T00:00:00"/>
+    <x v="7"/>
+    <n v="29137.15"/>
+    <n v="2110.85"/>
+    <n v="7.2445314658434332E-2"/>
+  </r>
+  <r>
+    <n v="14"/>
+    <n v="1586035"/>
+    <x v="1"/>
+    <d v="2026-08-26T00:00:00"/>
+    <x v="7"/>
+    <n v="731.65"/>
+    <n v="33.35"/>
+    <n v="4.5581903915806743E-2"/>
+  </r>
+  <r>
+    <n v="1"/>
+    <n v="1586037"/>
+    <x v="1"/>
+    <d v="2026-08-26T00:00:00"/>
+    <x v="7"/>
+    <n v="3121.87"/>
+    <n v="178.13"/>
+    <n v="5.7058750044044114E-2"/>
+  </r>
+  <r>
+    <n v="6"/>
+    <n v="1586038"/>
+    <x v="1"/>
+    <d v="2026-08-26T00:00:00"/>
+    <x v="7"/>
+    <n v="5714.59"/>
+    <n v="260.41000000000003"/>
+    <n v="4.5569323433527167E-2"/>
+  </r>
+  <r>
+    <n v="1"/>
+    <n v="1590857"/>
+    <x v="1"/>
+    <d v="2026-09-01T00:00:00"/>
+    <x v="9"/>
+    <n v="5719.81"/>
+    <n v="274.19"/>
+    <n v="4.7936906995162426E-2"/>
+  </r>
+  <r>
+    <n v="6"/>
+    <n v="1590855"/>
+    <x v="1"/>
+    <d v="2026-09-01T00:00:00"/>
+    <x v="9"/>
+    <n v="7233.26"/>
+    <n v="346.74"/>
+    <n v="4.7936891526089202E-2"/>
+  </r>
+  <r>
+    <n v="1"/>
+    <n v="1590856"/>
+    <x v="1"/>
+    <d v="2026-09-01T00:00:00"/>
+    <x v="9"/>
+    <n v="8950.94"/>
+    <n v="429.06"/>
+    <n v="4.7934630329328536E-2"/>
+  </r>
+  <r>
+    <n v="1"/>
+    <n v="1592968"/>
+    <x v="1"/>
+    <d v="2026-09-03T00:00:00"/>
+    <x v="9"/>
+    <n v="13038.84"/>
+    <n v="683.16"/>
+    <n v="5.2394231388681815E-2"/>
+  </r>
+  <r>
+    <n v="1"/>
+    <n v="1591866"/>
+    <x v="5"/>
+    <d v="2026-09-03T00:00:00"/>
+    <x v="9"/>
+    <n v="31263.87"/>
+    <n v="2115.33"/>
+    <n v="6.7660529550564272E-2"/>
+  </r>
+  <r>
+    <n v="1"/>
+    <n v="1600122"/>
+    <x v="1"/>
+    <d v="2026-09-15T00:00:00"/>
+    <x v="9"/>
+    <n v="713.58"/>
+    <n v="14.42"/>
+    <n v="2.0207965469884244E-2"/>
+  </r>
+  <r>
+    <n v="1"/>
+    <n v="1600120"/>
+    <x v="1"/>
+    <d v="2026-09-15T00:00:00"/>
+    <x v="9"/>
+    <n v="12416.42"/>
+    <n v="556.58000000000004"/>
+    <n v="4.4826125404907373E-2"/>
+  </r>
+  <r>
+    <n v="1"/>
+    <n v="1601195"/>
+    <x v="9"/>
+    <d v="2026-09-17T00:00:00"/>
+    <x v="9"/>
+    <n v="13793.56"/>
+    <n v="54.42"/>
+    <n v="3.9453194099275312E-3"/>
+  </r>
+  <r>
+    <n v="1"/>
+    <n v="1605495"/>
+    <x v="1"/>
+    <d v="2026-09-21T00:00:00"/>
+    <x v="9"/>
+    <n v="5943.64"/>
+    <n v="264.36"/>
+    <n v="4.4477794752037475E-2"/>
+  </r>
+  <r>
+    <n v="1"/>
+    <n v="1605711"/>
+    <x v="9"/>
+    <d v="2026-09-21T00:00:00"/>
+    <x v="9"/>
+    <n v="14124.06"/>
+    <n v="169.17"/>
+    <n v="1.1977434250491715E-2"/>
+  </r>
+  <r>
+    <n v="1"/>
+    <n v="1604678"/>
+    <x v="8"/>
+    <d v="2026-09-21T00:00:00"/>
+    <x v="9"/>
+    <n v="27635.57"/>
+    <n v="1525.38"/>
+    <n v="5.5196256129328984E-2"/>
+  </r>
+  <r>
+    <n v="1"/>
+    <n v="1605727"/>
+    <x v="5"/>
+    <d v="2026-09-21T00:00:00"/>
+    <x v="9"/>
+    <n v="112933.07"/>
+    <n v="8181.49"/>
+    <n v="7.2445475891162792E-2"/>
+  </r>
+  <r>
+    <n v="6"/>
+    <n v="1611752"/>
+    <x v="1"/>
+    <d v="2026-09-30T00:00:00"/>
+    <x v="9"/>
+    <n v="4055.13"/>
+    <n v="169.87"/>
+    <n v="4.1890149021116464E-2"/>
+  </r>
+  <r>
+    <n v="1"/>
+    <n v="1611750"/>
+    <x v="1"/>
+    <d v="2026-09-30T00:00:00"/>
+    <x v="9"/>
+    <n v="7224.66"/>
+    <n v="311.33999999999997"/>
+    <n v="4.3094069478702111E-2"/>
+  </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5D6E48F1-87EF-4E9B-AB74-BF2114D29F4E}" name="Tabela dinâmica7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16" rowHeaderCaption="Mês">
-  <location ref="A3:D11" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5D6E48F1-87EF-4E9B-AB74-BF2114D29F4E}" name="Tabela dinâmica7" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16" rowHeaderCaption="Mês">
+  <location ref="A3:D13" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" showAll="0">
-      <items count="8">
+      <items count="10">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
@@ -7092,6 +8752,8 @@
         <item x="4"/>
         <item x="5"/>
         <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -7102,7 +8764,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="8">
+  <rowItems count="10">
     <i>
       <x/>
     </i>
@@ -7123,6 +8785,12 @@
     </i>
     <i>
       <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
     </i>
     <i t="grand">
       <x/>
@@ -7175,7 +8843,7 @@
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="15" format="0" series="1">
+    <chartFormat chart="15" format="17" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -7184,7 +8852,7 @@
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="15" format="1" series="1">
+    <chartFormat chart="15" format="18" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -7193,7 +8861,91 @@
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="15" format="2" series="1">
+    <chartFormat chart="15" format="19">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="15" format="20">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="15" format="21">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="15" format="22">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="15" format="23">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="15" format="24">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="15" format="25">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="6"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="15" format="26" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -7202,7 +8954,31 @@
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="15" format="3">
+    <chartFormat chart="15" format="27">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="15" format="28">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="15" format="29">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -7214,31 +8990,7 @@
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="15" format="4">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="15" format="5">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="15" format="6">
+    <chartFormat chart="15" format="30">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -7250,7 +9002,7 @@
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="15" format="7">
+    <chartFormat chart="15" format="31">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -7262,7 +9014,7 @@
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="15" format="8">
+    <chartFormat chart="15" format="32">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -7274,7 +9026,7 @@
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="15" format="9">
+    <chartFormat chart="15" format="33">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -7282,90 +9034,6 @@
           </reference>
           <reference field="0" count="1" selected="0">
             <x v="6"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="15" format="10">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="15" format="11">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="15" format="12">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="15" format="13">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="15" format="14">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="6"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="15" format="15">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="5"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="15" format="16">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="4"/>
           </reference>
         </references>
       </pivotArea>
@@ -7384,46 +9052,49 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D881F340-3154-4F0A-8D10-4A2CAE3AAF32}" name="Tabela dinâmica13" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" chartFormat="31" rowHeaderCaption="Fornecedores ">
-  <location ref="A4:D13" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D881F340-3154-4F0A-8D10-4A2CAE3AAF32}" name="Tabela dinâmica13" cacheId="19" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" chartFormat="31" rowHeaderCaption="Fornecedores ">
+  <location ref="A4:D15" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="8">
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
-      <items count="28">
+      <items count="31">
+        <item m="1" x="27"/>
+        <item m="1" x="26"/>
+        <item m="1" x="28"/>
+        <item m="1" x="21"/>
+        <item m="1" x="23"/>
+        <item m="1" x="22"/>
         <item m="1" x="24"/>
-        <item m="1" x="23"/>
         <item m="1" x="25"/>
+        <item m="1" x="29"/>
+        <item m="1" x="17"/>
         <item m="1" x="18"/>
+        <item m="1" x="19"/>
         <item m="1" x="20"/>
-        <item m="1" x="19"/>
-        <item m="1" x="21"/>
-        <item m="1" x="22"/>
-        <item m="1" x="26"/>
-        <item m="1" x="14"/>
+        <item m="1" x="16"/>
+        <item sd="0" x="0"/>
+        <item m="1" x="11"/>
         <item m="1" x="15"/>
-        <item m="1" x="16"/>
-        <item m="1" x="17"/>
-        <item m="1" x="13"/>
-        <item sd="0" x="0"/>
-        <item m="1" x="8"/>
-        <item m="1" x="12"/>
         <item sd="0" x="1"/>
         <item sd="0" x="2"/>
         <item sd="0" x="3"/>
         <item sd="0" x="4"/>
         <item sd="0" x="5"/>
-        <item m="1" x="11"/>
+        <item m="1" x="14"/>
         <item sd="0" x="6"/>
+        <item m="1" x="13"/>
+        <item m="1" x="12"/>
+        <item sd="0" x="7"/>
+        <item x="8"/>
+        <item x="9"/>
         <item m="1" x="10"/>
-        <item m="1" x="9"/>
-        <item sd="0" x="7"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField numFmtId="14" multipleItemSelectionAllowed="1" showAll="0"/>
     <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="8">
+      <items count="11">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
@@ -7431,6 +9102,9 @@
         <item x="4"/>
         <item x="5"/>
         <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -7441,7 +9115,7 @@
   <rowFields count="1">
     <field x="2"/>
   </rowFields>
-  <rowItems count="9">
+  <rowItems count="11">
     <i>
       <x v="14"/>
     </i>
@@ -7465,6 +9139,12 @@
     </i>
     <i>
       <x v="26"/>
+    </i>
+    <i>
+      <x v="27"/>
+    </i>
+    <i>
+      <x v="28"/>
     </i>
     <i t="grand">
       <x/>
@@ -7493,7 +9173,7 @@
     <dataField name="Média de Ganha por %" fld="7" subtotal="average" baseField="2" baseItem="14" numFmtId="10"/>
   </dataFields>
   <formats count="29">
-    <format dxfId="28">
+    <format dxfId="57">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -7502,7 +9182,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="27">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -7511,7 +9191,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="26">
+    <format dxfId="55">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -7520,7 +9200,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="25">
+    <format dxfId="54">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -7529,37 +9209,37 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="24">
+    <format dxfId="53">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="23">
+    <format dxfId="52">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="22">
+    <format dxfId="51">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="21">
+    <format dxfId="50">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="20">
+    <format dxfId="49">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
+    <format dxfId="48">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="18">
+    <format dxfId="47">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="2">
@@ -7569,19 +9249,19 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
+    <format dxfId="46">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="16">
+    <format dxfId="45">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="15">
+    <format dxfId="44">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="14">
+    <format dxfId="43">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
+    <format dxfId="42">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="3">
@@ -7592,7 +9272,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="12">
+    <format dxfId="41">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -7601,7 +9281,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="11">
+    <format dxfId="40">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -7610,7 +9290,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="39">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -7619,7 +9299,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="9">
+    <format dxfId="38">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -7628,29 +9308,29 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="8">
+    <format dxfId="37">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="7">
+    <format dxfId="36">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="35">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="5">
+    <format dxfId="34">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="4">
+    <format dxfId="33">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="3">
+    <format dxfId="32">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="2">
+    <format dxfId="31">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="3">
@@ -7661,10 +9341,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="30">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisPage" fieldPosition="0"/>
     </format>
-    <format dxfId="0">
+    <format dxfId="29">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisPage" fieldPosition="0"/>
     </format>
   </formats>
@@ -7701,17 +9381,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C2E36174-8176-4BFA-A85A-B4B760440A70}" name="Tabela1" displayName="Tabela1" ref="A1:H116" totalsRowShown="0" headerRowDxfId="45" headerRowCellStyle="Moeda">
-  <autoFilter ref="A1:H116" xr:uid="{C2E36174-8176-4BFA-A85A-B4B760440A70}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C2E36174-8176-4BFA-A85A-B4B760440A70}" name="Tabela1" displayName="Tabela1" ref="A1:H130" totalsRowShown="0" headerRowDxfId="74" headerRowCellStyle="Moeda">
+  <autoFilter ref="A1:H130" xr:uid="{C2E36174-8176-4BFA-A85A-B4B760440A70}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{E43F716C-17FB-403E-A60C-9039879F6326}" name="L.P" dataDxfId="44" totalsRowDxfId="43"/>
-    <tableColumn id="2" xr3:uid="{BFD5FD24-83B9-439A-AFE7-87F024B9F391}" name="Duplicata" dataDxfId="42" totalsRowDxfId="41"/>
-    <tableColumn id="3" xr3:uid="{FC99EE4A-E72D-40EC-A5A7-C45C6E6E3FC0}" name="Favorecido" dataDxfId="40" totalsRowDxfId="39"/>
-    <tableColumn id="4" xr3:uid="{4A48BFFC-F963-44D0-892A-A37B6B103A64}" name="Vencimento" dataDxfId="38" totalsRowDxfId="37"/>
-    <tableColumn id="9" xr3:uid="{9160D380-BAF1-4759-895D-0955385C2CBD}" name="Mês" dataDxfId="36" totalsRowDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{2C991543-7C1B-4E66-9DD9-1DCBA69EACC7}" name="Valor líquido" dataDxfId="34" totalsRowDxfId="33" dataCellStyle="Moeda"/>
-    <tableColumn id="6" xr3:uid="{15C6E1F5-CE2D-4912-9957-34BA57A7541E}" name="Desconto Financeiro" dataDxfId="32" totalsRowDxfId="31" dataCellStyle="Moeda"/>
-    <tableColumn id="7" xr3:uid="{C7BEA4B3-11CA-417D-A976-DB09212BCA5D}" name="Ganha por %" dataDxfId="30" totalsRowDxfId="29" dataCellStyle="Porcentagem">
+    <tableColumn id="1" xr3:uid="{E43F716C-17FB-403E-A60C-9039879F6326}" name="L.P" dataDxfId="73" totalsRowDxfId="72"/>
+    <tableColumn id="2" xr3:uid="{BFD5FD24-83B9-439A-AFE7-87F024B9F391}" name="Duplicata" dataDxfId="71" totalsRowDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{FC99EE4A-E72D-40EC-A5A7-C45C6E6E3FC0}" name="Favorecido" dataDxfId="69" totalsRowDxfId="68"/>
+    <tableColumn id="4" xr3:uid="{4A48BFFC-F963-44D0-892A-A37B6B103A64}" name="Vencimento" dataDxfId="67" totalsRowDxfId="66"/>
+    <tableColumn id="9" xr3:uid="{9160D380-BAF1-4759-895D-0955385C2CBD}" name="Mês" dataDxfId="65" totalsRowDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{2C991543-7C1B-4E66-9DD9-1DCBA69EACC7}" name="Valor líquido" dataDxfId="63" totalsRowDxfId="62" dataCellStyle="Moeda"/>
+    <tableColumn id="6" xr3:uid="{15C6E1F5-CE2D-4912-9957-34BA57A7541E}" name="Desconto Financeiro" dataDxfId="61" totalsRowDxfId="60" dataCellStyle="Moeda"/>
+    <tableColumn id="7" xr3:uid="{C7BEA4B3-11CA-417D-A976-DB09212BCA5D}" name="Ganha por %" dataDxfId="59" totalsRowDxfId="58" dataCellStyle="Porcentagem">
       <calculatedColumnFormula>G2/F2</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -8036,11 +9716,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{310DA7BC-6D6C-47EB-90B7-5DE8A3716D54}">
-  <dimension ref="A3:D11"/>
+  <dimension ref="A3:D13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -8159,16 +9839,44 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="17">
+        <v>232778.93999999997</v>
+      </c>
+      <c r="C11" s="17">
+        <v>5529.87</v>
+      </c>
+      <c r="D11" s="18">
+        <v>3.603415173702252E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="17">
+        <v>11041.27</v>
+      </c>
+      <c r="C12" s="17">
+        <v>436.23</v>
+      </c>
+      <c r="D12" s="18">
+        <v>3.6166276882344799E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="17">
-        <v>816185.36000000045</v>
-      </c>
-      <c r="C11" s="17">
-        <v>25849.740000000013</v>
-      </c>
-      <c r="D11" s="18">
-        <v>4.0429820783346337E-2</v>
+      <c r="B13" s="17">
+        <v>1060005.5700000008</v>
+      </c>
+      <c r="C13" s="17">
+        <v>31815.840000000011</v>
+      </c>
+      <c r="D13" s="18">
+        <v>3.9901589341810678E-2</v>
       </c>
     </row>
   </sheetData>
@@ -8179,11 +9887,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A10B5FA-6D15-45AC-BC0B-8204D62EE5BF}">
-  <dimension ref="A2:E13"/>
+  <dimension ref="A2:E16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="68.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23.77734375" bestFit="1" customWidth="1"/>
   </cols>
@@ -8230,13 +9938,13 @@
         <v>15</v>
       </c>
       <c r="B6" s="30">
-        <v>212410.12000000005</v>
+        <v>298315.78000000003</v>
       </c>
       <c r="C6" s="30">
-        <v>9645.380000000001</v>
+        <v>13603.220000000001</v>
       </c>
       <c r="D6" s="31">
-        <v>4.3854667932527111E-2</v>
+        <v>4.3425467679551071E-2</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.35">
@@ -8272,13 +9980,13 @@
         <v>16</v>
       </c>
       <c r="B9" s="30">
-        <v>148813.76999999999</v>
+        <v>168020.38999999998</v>
       </c>
       <c r="C9" s="30">
-        <v>2390.5</v>
+        <v>2995.26</v>
       </c>
       <c r="D9" s="31">
-        <v>1.5904992681468083E-2</v>
+        <v>1.850200393300758E-2</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.35">
@@ -8286,13 +9994,13 @@
         <v>17</v>
       </c>
       <c r="B10" s="30">
-        <v>219380.20999999996</v>
+        <v>539254.35</v>
       </c>
       <c r="C10" s="30">
-        <v>5504.3899999999994</v>
+        <v>19760.41</v>
       </c>
       <c r="D10" s="31">
-        <v>2.1831772351583293E-2</v>
+        <v>3.5396597665174945E-2</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.35">
@@ -8325,18 +10033,47 @@
     </row>
     <row r="13" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="A13" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="30">
+        <v>55962.58</v>
+      </c>
+      <c r="C13" s="30">
+        <v>2019.4</v>
+      </c>
+      <c r="D13" s="31">
+        <v>3.6318074151455861E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="A14" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="30">
+        <v>27917.62</v>
+      </c>
+      <c r="C14" s="30">
+        <v>223.58999999999997</v>
+      </c>
+      <c r="D14" s="31">
+        <v>7.9613768302096224E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="A15" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="32">
-        <v>816185.36</v>
-      </c>
-      <c r="C13" s="32">
-        <v>25849.74</v>
-      </c>
-      <c r="D13" s="33">
-        <v>4.0429820783346351E-2</v>
-      </c>
-    </row>
+      <c r="B15" s="32">
+        <v>1325051.9800000002</v>
+      </c>
+      <c r="C15" s="32">
+        <v>46911.349999999991</v>
+      </c>
+      <c r="D15" s="33">
+        <v>4.0237260107795457E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
@@ -8344,7 +10081,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H116"/>
+  <dimension ref="A1:H130"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.5546875" customWidth="1"/>
@@ -11486,6 +13223,384 @@
       <c r="H116" s="7">
         <f t="shared" si="16"/>
         <v>4.5569323433527167E-2</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A117" s="1">
+        <v>1</v>
+      </c>
+      <c r="B117" s="2">
+        <v>1590857</v>
+      </c>
+      <c r="C117" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="D117" s="3">
+        <v>46266</v>
+      </c>
+      <c r="E117" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F117" s="4">
+        <v>5719.81</v>
+      </c>
+      <c r="G117" s="4">
+        <v>274.19</v>
+      </c>
+      <c r="H117" s="7">
+        <f>G117/F117</f>
+        <v>4.7936906995162426E-2</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A118" s="1">
+        <v>6</v>
+      </c>
+      <c r="B118" s="2">
+        <v>1590855</v>
+      </c>
+      <c r="C118" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="D118" s="3">
+        <v>46266</v>
+      </c>
+      <c r="E118" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F118" s="4">
+        <v>7233.26</v>
+      </c>
+      <c r="G118" s="4">
+        <v>346.74</v>
+      </c>
+      <c r="H118" s="7">
+        <f>G118/F118</f>
+        <v>4.7936891526089202E-2</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A119" s="1">
+        <v>1</v>
+      </c>
+      <c r="B119" s="2">
+        <v>1590856</v>
+      </c>
+      <c r="C119" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="D119" s="3">
+        <v>46266</v>
+      </c>
+      <c r="E119" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F119" s="13">
+        <v>8950.94</v>
+      </c>
+      <c r="G119" s="13">
+        <v>429.06</v>
+      </c>
+      <c r="H119" s="14">
+        <f>G119/F119</f>
+        <v>4.7934630329328536E-2</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A120" s="1">
+        <v>1</v>
+      </c>
+      <c r="B120" s="2">
+        <v>1592968</v>
+      </c>
+      <c r="C120" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="D120" s="3">
+        <v>46268</v>
+      </c>
+      <c r="E120" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F120" s="4">
+        <v>13038.84</v>
+      </c>
+      <c r="G120" s="4">
+        <v>683.16</v>
+      </c>
+      <c r="H120" s="7">
+        <f>G120/F120</f>
+        <v>5.2394231388681815E-2</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A121" s="1">
+        <v>1</v>
+      </c>
+      <c r="B121" s="2">
+        <v>1591866</v>
+      </c>
+      <c r="C121" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="D121" s="3">
+        <v>46268</v>
+      </c>
+      <c r="E121" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F121" s="4">
+        <v>31263.87</v>
+      </c>
+      <c r="G121" s="4">
+        <v>2115.33</v>
+      </c>
+      <c r="H121" s="7">
+        <f>G121/F121</f>
+        <v>6.7660529550564272E-2</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A122" s="1">
+        <v>1</v>
+      </c>
+      <c r="B122" s="2">
+        <v>1600122</v>
+      </c>
+      <c r="C122" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="D122" s="3">
+        <v>46280</v>
+      </c>
+      <c r="E122" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F122" s="4">
+        <v>713.58</v>
+      </c>
+      <c r="G122" s="4">
+        <v>14.42</v>
+      </c>
+      <c r="H122" s="7">
+        <f>G122/F122</f>
+        <v>2.0207965469884244E-2</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A123" s="1">
+        <v>1</v>
+      </c>
+      <c r="B123" s="2">
+        <v>1600120</v>
+      </c>
+      <c r="C123" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="D123" s="3">
+        <v>46280</v>
+      </c>
+      <c r="E123" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F123" s="4">
+        <v>12416.42</v>
+      </c>
+      <c r="G123" s="4">
+        <v>556.58000000000004</v>
+      </c>
+      <c r="H123" s="7">
+        <f>G123/F123</f>
+        <v>4.4826125404907373E-2</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A124" s="1">
+        <v>1</v>
+      </c>
+      <c r="B124" s="2">
+        <v>1601195</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D124" s="3">
+        <v>46282</v>
+      </c>
+      <c r="E124" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F124" s="4">
+        <v>13793.56</v>
+      </c>
+      <c r="G124" s="4">
+        <v>54.42</v>
+      </c>
+      <c r="H124" s="7">
+        <f>G124/F124</f>
+        <v>3.9453194099275312E-3</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A125" s="1">
+        <v>1</v>
+      </c>
+      <c r="B125" s="2">
+        <v>1605495</v>
+      </c>
+      <c r="C125" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="D125" s="3">
+        <v>46286</v>
+      </c>
+      <c r="E125" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F125" s="4">
+        <v>5943.64</v>
+      </c>
+      <c r="G125" s="4">
+        <v>264.36</v>
+      </c>
+      <c r="H125" s="7">
+        <f>G125/F125</f>
+        <v>4.4477794752037475E-2</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A126" s="1">
+        <v>1</v>
+      </c>
+      <c r="B126" s="2">
+        <v>1605711</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D126" s="3">
+        <v>46286</v>
+      </c>
+      <c r="E126" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F126" s="4">
+        <v>14124.06</v>
+      </c>
+      <c r="G126" s="4">
+        <v>169.17</v>
+      </c>
+      <c r="H126" s="7">
+        <f>G126/F126</f>
+        <v>1.1977434250491715E-2</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A127" s="1">
+        <v>1</v>
+      </c>
+      <c r="B127" s="2">
+        <v>1604678</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D127" s="3">
+        <v>46286</v>
+      </c>
+      <c r="E127" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F127" s="4">
+        <v>27635.57</v>
+      </c>
+      <c r="G127" s="4">
+        <v>1525.38</v>
+      </c>
+      <c r="H127" s="7">
+        <f>G127/F127</f>
+        <v>5.5196256129328984E-2</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A128" s="1">
+        <v>1</v>
+      </c>
+      <c r="B128" s="2">
+        <v>1605727</v>
+      </c>
+      <c r="C128" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="D128" s="3">
+        <v>46286</v>
+      </c>
+      <c r="E128" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F128" s="4">
+        <v>112933.07</v>
+      </c>
+      <c r="G128" s="4">
+        <v>8181.49</v>
+      </c>
+      <c r="H128" s="7">
+        <f>G128/F128</f>
+        <v>7.2445475891162792E-2</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A129" s="1">
+        <v>6</v>
+      </c>
+      <c r="B129" s="2">
+        <v>1611752</v>
+      </c>
+      <c r="C129" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="D129" s="3">
+        <v>46295</v>
+      </c>
+      <c r="E129" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F129" s="4">
+        <v>4055.13</v>
+      </c>
+      <c r="G129" s="4">
+        <v>169.87</v>
+      </c>
+      <c r="H129" s="7">
+        <f>G129/F129</f>
+        <v>4.1890149021116464E-2</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A130" s="1">
+        <v>1</v>
+      </c>
+      <c r="B130" s="2">
+        <v>1611750</v>
+      </c>
+      <c r="C130" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="D130" s="3">
+        <v>46295</v>
+      </c>
+      <c r="E130" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F130" s="13">
+        <v>7224.66</v>
+      </c>
+      <c r="G130" s="13">
+        <v>311.33999999999997</v>
+      </c>
+      <c r="H130" s="14">
+        <f>G130/F130</f>
+        <v>4.3094069478702111E-2</v>
       </c>
     </row>
   </sheetData>
@@ -11837,15 +13952,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="00214df3-eeab-40e9-9d54-728e38b1ce7f" xsi:nil="true"/>
@@ -11856,19 +13962,35 @@
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D919D950-698A-4A4D-9E20-C78F9D115B9D}"/>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{395444AC-F904-4087-861B-5E7FF9660FE2}">
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D919D950-698A-4A4D-9E20-C78F9D115B9D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="52079a64-9187-4293-860a-cd501a0368c7"/>
+    <ds:schemaRef ds:uri="00214df3-eeab-40e9-9d54-728e38b1ce7f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CDDE870-10C7-4BE9-834C-0469A4A93DFA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -11877,4 +13999,12 @@
     <ds:schemaRef ds:uri="52079a64-9187-4293-860a-cd501a0368c7"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{395444AC-F904-4087-861B-5E7FF9660FE2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>